<commit_message>
Shivers: Schwarz ab Takt 44,5, Blinder in Chorus 1b schnell ein und bis Takt 46 aus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/Shivers_v1/quelle/struktur.xlsx
+++ b/songs/Shivers_v1/quelle/struktur.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18420" yWindow="3828" windowWidth="27240" windowHeight="20436" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18420" yWindow="10488" windowWidth="27240" windowHeight="13776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Struktur" sheetId="1" state="visible" r:id="rId1"/>
@@ -2348,7 +2348,7 @@
       <c r="G149" s="5" t="n"/>
       <c r="H149" s="6" t="n"/>
     </row>
-    <row r="150" collapsed="1" ht="28.8" customHeight="1">
+    <row r="150" ht="28.8" customHeight="1">
       <c r="A150" s="4" t="n">
         <v>37</v>
       </c>
@@ -2361,7 +2361,8 @@
         <is>
           <t>SCENE_STAR, Farben SCHEME_NEON
 Ausgabe: Blinder bei 0 ms, 909 ms lang
-Drehender Stern in Neon-Farben, Farbwechsel im Beat. Auf den Einsatz springt ein Blinder auf (warmweiß, alle Geräte) und klingt über 2 Beats ab.</t>
+Schluss (1 Beats): progBlack(455, 10), Farben SCHEME_NEON
+Drehender Stern in Neon-Farben, Farbwechsel im Beat. Auf den Einsatz springt ein Blinder auf (warmweiß, alle Geräte) und klingt über 2 Beats ab. Ab Takt 44,5 ist es schon schwarz.</t>
         </is>
       </c>
       <c r="D150" s="6" t="n"/>
@@ -2377,7 +2378,7 @@
         </is>
       </c>
     </row>
-    <row r="151" hidden="1" outlineLevel="2">
+    <row r="151" outlineLevel="2">
       <c r="A151" s="4" t="n">
         <v>37.25</v>
       </c>
@@ -2389,7 +2390,7 @@
       <c r="G151" s="5" t="n"/>
       <c r="H151" s="6" t="n"/>
     </row>
-    <row r="152" hidden="1" outlineLevel="2">
+    <row r="152" outlineLevel="2">
       <c r="A152" s="4" t="n">
         <v>37.5</v>
       </c>
@@ -2401,7 +2402,7 @@
       <c r="G152" s="5" t="n"/>
       <c r="H152" s="6" t="n"/>
     </row>
-    <row r="153" hidden="1" outlineLevel="2">
+    <row r="153" outlineLevel="2">
       <c r="A153" s="4" t="n">
         <v>37.75</v>
       </c>
@@ -2413,7 +2414,7 @@
       <c r="G153" s="5" t="n"/>
       <c r="H153" s="6" t="n"/>
     </row>
-    <row r="154" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="154" outlineLevel="1" collapsed="1">
       <c r="A154" s="4" t="n">
         <v>38</v>
       </c>
@@ -2461,7 +2462,7 @@
       <c r="G157" s="5" t="n"/>
       <c r="H157" s="6" t="n"/>
     </row>
-    <row r="158" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="158" outlineLevel="1" collapsed="1">
       <c r="A158" s="4" t="n">
         <v>39</v>
       </c>
@@ -2509,7 +2510,7 @@
       <c r="G161" s="5" t="n"/>
       <c r="H161" s="6" t="n"/>
     </row>
-    <row r="162" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="162" outlineLevel="1" collapsed="1">
       <c r="A162" s="4" t="n">
         <v>40</v>
       </c>
@@ -2557,7 +2558,7 @@
       <c r="G165" s="5" t="n"/>
       <c r="H165" s="6" t="n"/>
     </row>
-    <row r="166" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="166" outlineLevel="1" collapsed="1">
       <c r="A166" s="4" t="n">
         <v>41</v>
       </c>
@@ -2605,7 +2606,7 @@
       <c r="G169" s="5" t="n"/>
       <c r="H169" s="6" t="n"/>
     </row>
-    <row r="170" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="170" outlineLevel="1" collapsed="1">
       <c r="A170" s="4" t="n">
         <v>42</v>
       </c>
@@ -2653,7 +2654,7 @@
       <c r="G173" s="5" t="n"/>
       <c r="H173" s="6" t="n"/>
     </row>
-    <row r="174" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="174" outlineLevel="1" collapsed="1">
       <c r="A174" s="4" t="n">
         <v>43</v>
       </c>
@@ -2701,7 +2702,7 @@
       <c r="G177" s="5" t="n"/>
       <c r="H177" s="6" t="n"/>
     </row>
-    <row r="178" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="178" outlineLevel="1">
       <c r="A178" s="4" t="n">
         <v>44</v>
       </c>
@@ -2713,7 +2714,7 @@
       <c r="G178" s="5" t="n"/>
       <c r="H178" s="6" t="n"/>
     </row>
-    <row r="179" hidden="1" outlineLevel="2">
+    <row r="179" outlineLevel="2">
       <c r="A179" s="4" t="n">
         <v>44.25</v>
       </c>
@@ -2725,13 +2726,21 @@
       <c r="G179" s="5" t="n"/>
       <c r="H179" s="6" t="n"/>
     </row>
-    <row r="180" hidden="1" outlineLevel="2">
+    <row r="180" outlineLevel="2">
       <c r="A180" s="4" t="n">
         <v>44.5</v>
       </c>
       <c r="B180" s="5" t="n"/>
-      <c r="C180" s="6" t="n"/>
-      <c r="D180" s="6" t="n"/>
+      <c r="C180" s="6" t="inlineStr">
+        <is>
+          <t>ab hier schon Schwarz (1 Beat vor der mini pause)</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>ab hier schon progBlack</t>
+        </is>
+      </c>
       <c r="E180" s="6" t="n"/>
       <c r="F180" s="5" t="n"/>
       <c r="G180" s="5" t="n"/>
@@ -2748,9 +2757,9 @@
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>progBlack(909, 10), Farben SCHEME_SUNSET
-Ausgabe: Blinder von 'Chorus 1b' blendet in den letzten 455 ms ein
-2 Beats Schwarz; darin blendet der starke Blinder für den Wiedereinsatz (Takt 45,25) ein.</t>
+          <t>progBlack(909, 11), Farben SCHEME_SUNSET
+Ausgabe: Blinder von 'Chorus 1b' blendet in den letzten 45 ms ein
+2 Beats Schwarz bis zum Wiedereinsatz auf Takt 45,25.</t>
         </is>
       </c>
       <c r="D181" s="6" t="n"/>
@@ -2790,11 +2799,15 @@
       <c r="C183" s="6" t="inlineStr">
         <is>
           <t>SCENE_SPARKLE, Farben SCHEME_NEON
-Ausgabe: Blinder voll bei 0 ms, 1364 ms lang, Blinder blendet in den 455 ms davor ein, 0 ms voll, 909 ms aus
-Schnelle Einzelblitze in Pink, Cyan, Violett. Ein starker Blinder blendet im letzten Beat der Pause ein, ist auf dem Wiedereinsatz voll hell und klingt über 2 Beats ab.</t>
-        </is>
-      </c>
-      <c r="D183" s="6" t="n"/>
+Ausgabe: Blinder voll bei 0 ms, 1409 ms lang, Blinder blendet in den 45 ms davor ein, 0 ms voll, 1364 ms aus
+Schnelle Einzelblitze in Pink, Cyan, Violett. Ein starker Blinder blendet ganz kurz vor dem Wiedereinsatz ein, ist auf Takt 45,25 voll hell und klingt bis Takt 46 (3 Beats) aus.</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>den Blinder erst auf 45,25 -&gt; sehr schnell einblenden und bis 46,0 ausfaden</t>
+        </is>
+      </c>
       <c r="E183" s="6" t="n"/>
       <c r="F183" s="5" t="n"/>
       <c r="G183" s="5">
@@ -3178,7 +3191,7 @@
       </c>
       <c r="C214" s="6" t="inlineStr">
         <is>
-          <t>progBeatColors(14545, 12, 132, 2, false), Farben SCHEME_SUNSET
+          <t>progBeatColors(14545, 13, 132, 2, false), Farben SCHEME_SUNSET
 Ausgabe: Farbwechsel weich (100 % des Schritts)
 Die ganze Bühne leuchtet in einer Sunset-Farbe und fließt alle 2 Beats weich in die nächste.</t>
         </is>
@@ -4735,7 +4748,7 @@
       </c>
       <c r="C338" s="6" t="inlineStr">
         <is>
-          <t>progBlack(909, 17), Farben SCHEME_SUNSET
+          <t>progBlack(909, 18), Farben SCHEME_SUNSET
 Schluss (2 Beats): SCENE_COLORS, Farben SCHEME_WHITE
    Ausgabe: Tor 4x pro Beat, 50 % hell
 2 Beats Schwarz, ab Takt 84,5 weißer Strobo im Takt (4 Blitze pro Beat) auf allen Geräten.</t>
@@ -4776,11 +4789,7 @@
           <t>erst hier der weiße Strobo (4 Blitze pro Beat), davor 2 Beats Schwarz</t>
         </is>
       </c>
-      <c r="D340" s="6" t="inlineStr">
-        <is>
-          <t>hier erst der strobo</t>
-        </is>
-      </c>
+      <c r="D340" s="6" t="n"/>
       <c r="E340" s="6" t="n"/>
       <c r="F340" s="5" t="n"/>
       <c r="G340" s="5" t="n"/>
@@ -4827,7 +4836,7 @@
         </is>
       </c>
     </row>
-    <row r="343" outlineLevel="2">
+    <row r="343" outlineLevel="2" ht="28.8" customHeight="1">
       <c r="A343" s="4" t="n">
         <v>85.25</v>
       </c>
@@ -4837,11 +4846,7 @@
           <t>Höhepunkt des Blinders erst hier: blendet ab Takt 85 über 1 Beat ein, klingt danach über 2 Beats ab</t>
         </is>
       </c>
-      <c r="D343" s="6" t="inlineStr">
-        <is>
-          <t>hier erst höhepunkt des Blinders</t>
-        </is>
-      </c>
+      <c r="D343" s="6" t="n"/>
       <c r="E343" s="6" t="n"/>
       <c r="F343" s="5" t="n"/>
       <c r="G343" s="5" t="n"/>
@@ -6022,16 +6027,12 @@
         <is>
           <t>SCENE_FIRE, Farben SCHEME_RED
 Ausgabe: Übergang fade 455 ms, blendet die letzten 1818 ms aus
-Schluss (4 Beats): progBlack(1818, 23), Farben SCHEME_RED
+Schluss (4 Beats): progBlack(1818, 24), Farben SCHEME_RED
    Ausgabe: Blinder von 'Chorus 1 (3)' blendet in den letzten 909 ms ein
 Das rote Feuer aus 'you burn' blendet ganz langsam über einen Takt nach Schwarz aus, danach Stille; in den letzten 2 Beats blendet ein Blinder ein, voll hell auf dem Chorus-Einsatz (Takt 111).</t>
         </is>
       </c>
-      <c r="D438" s="6" t="inlineStr">
-        <is>
-          <t>hier bitte ganz langsam den ausfaden  über einen takt</t>
-        </is>
-      </c>
+      <c r="D438" s="6" t="n"/>
       <c r="E438" s="6" t="n"/>
       <c r="F438" s="5" t="n"/>
       <c r="G438" s="5">
@@ -6409,7 +6410,7 @@
       <c r="G467" s="5" t="n"/>
       <c r="H467" s="6" t="n"/>
     </row>
-    <row r="468" collapsed="1" ht="28.8" customHeight="1">
+    <row r="468" ht="28.8" customHeight="1">
       <c r="A468" s="4" t="n">
         <v>116.5</v>
       </c>
@@ -6420,7 +6421,7 @@
       </c>
       <c r="C468" s="6" t="inlineStr">
         <is>
-          <t>progBlack(1364, 25), Farben SCHEME_SUNSET
+          <t>progBlack(1364, 26), Farben SCHEME_SUNSET
 Ausgabe: Blinder bei 0 ms, 1364 ms lang, Blinder blendet 0 ms ein, 1318 ms voll, 46 ms aus
 Starker Blinder (warmweiß, alle Geräte) steht die ganzen 3 Beats voll bis zum Einsatz auf Takt 117,25.</t>
         </is>
@@ -6460,11 +6461,7 @@
           <t>Chorus 1b (3) beginnt jetzt erst auf Takt 117,25 (Part in der Tabelle verschoben); der Blinder steht bis dahin voll</t>
         </is>
       </c>
-      <c r="D470" s="6" t="inlineStr">
-        <is>
-          <t>etwas zu früh -&gt; erst bei 117,25 wieder hiermit einsteigen</t>
-        </is>
-      </c>
+      <c r="D470" s="6" t="n"/>
       <c r="E470" s="6" t="n"/>
       <c r="F470" s="5" t="n"/>
       <c r="G470" s="5">
@@ -6477,7 +6474,7 @@
         </is>
       </c>
     </row>
-    <row r="471">
+    <row r="471" ht="187.2" customHeight="1">
       <c r="A471" s="4" t="n">
         <v>117.25</v>
       </c>
@@ -6493,11 +6490,7 @@
 Schnelle Einzelblitze in Rot, Orange, Gelb, Einsatz auf Takt 117,25. Drei kurze Blinder auf den Vierteln 120,5 / 120,75 / 121. Am Schluss drei Blinder triolisch (124 / 124,33 / 124,66); der letzte bleibt voll hell und klingt über 2 Takte ins Schluss-Schwarz aus.</t>
         </is>
       </c>
-      <c r="D471" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">erst hier wieder einsteigen </t>
-        </is>
-      </c>
+      <c r="D471" s="6" t="n"/>
       <c r="E471" s="6" t="n"/>
       <c r="F471" s="5" t="n"/>
       <c r="G471" s="5" t="n"/>
@@ -6657,11 +6650,7 @@
           <t>drei kurze Blinder auf 120,5 / 120,75 / 121 (bleiben wie sie sind)</t>
         </is>
       </c>
-      <c r="D484" s="6" t="inlineStr">
-        <is>
-          <t>hier sind 3 blinder, sind ok und könnmen hier bleiben</t>
-        </is>
-      </c>
+      <c r="D484" s="6" t="n"/>
       <c r="E484" s="6" t="n"/>
       <c r="F484" s="5" t="n"/>
       <c r="G484" s="5" t="n"/>
@@ -6833,11 +6822,7 @@
           <t>drei Blinder triolisch auf 124 / 124,33 / 124,66; der letzte steht bis zum Songende voll und klingt dann über 2 Takte (3,6 s) ins Schluss-Schwarz aus</t>
         </is>
       </c>
-      <c r="D498" s="6" t="inlineStr">
-        <is>
-          <t>hier müssten noch mal drei blinder hin, aber triolisch, also bei 124,0, 124,33, 124, 66. der letzte blinder bei 124,66 soll dann über 2 takte ausfaden</t>
-        </is>
-      </c>
+      <c r="D498" s="6" t="n"/>
       <c r="E498" s="6" t="n"/>
       <c r="F498" s="5" t="n"/>
       <c r="G498" s="5" t="n"/>

</xml_diff>